<commit_message>
mis a jour manuellement PVT et DTO
</commit_message>
<xml_diff>
--- a/pvt_list.xlsx
+++ b/pvt_list.xlsx
@@ -1,30 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Dossier LOUMA\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_46CBBBEB4BD4E64F51C9DC61FC2C65EABA356C5E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE8C612E-D71E-46E2-9297-A76DBD35E99B}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
   <si>
     <t>DRV</t>
   </si>
@@ -39,6 +51,9 @@
   </si>
   <si>
     <t>PVT TEKNICOM CONSULTING GROUPE (SADI RUFISQUE-DIAMNIADIO)</t>
+  </si>
+  <si>
+    <t>IBRAHIMA SENE(SADI ZPPG)</t>
   </si>
   <si>
     <t>DRC</t>
@@ -89,8 +104,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -102,6 +117,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -139,18 +160,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -430,15 +452,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="58.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -449,7 +471,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -460,113 +482,124 @@
         <v>774981290</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="15">
       <c r="A3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="3">
+        <v>776647468</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15">
+      <c r="A4" s="4" t="s">
         <v>6</v>
-      </c>
-      <c r="C3" s="3">
-        <v>775499999</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
-        <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
+        <v>775499999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15">
+      <c r="A5" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2">
         <v>775945699</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2" t="s">
+    <row r="6" spans="1:3" ht="15">
+      <c r="A6" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="C5" s="3">
-        <v>776247047</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="4" t="s">
-        <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="3">
+        <v>776247047</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15">
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="2">
         <v>776665352</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
+    <row r="8" spans="1:3" ht="15">
+      <c r="A8" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="C7" s="3">
-        <v>775499999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="4" t="s">
-        <v>11</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="3">
+        <v>775499999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="15">
+      <c r="A9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="2">
         <v>781287163</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="2" t="s">
+    <row r="10" spans="1:3" ht="15">
+      <c r="A10" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="C9" s="2">
-        <v>772579898</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="2">
+        <v>772579898</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="15">
+      <c r="A11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="3">
         <v>774317541</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="2" t="s">
+    <row r="12" spans="1:3" ht="15">
+      <c r="A12" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="C11" s="3">
-        <v>773316647</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
-        <v>17</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="3">
+        <v>773316647</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15">
+      <c r="A13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="2">
         <v>775451818</v>
       </c>
     </row>

</xml_diff>

<commit_message>
garde moi  cette version du reporting mensuel qui marche bien
</commit_message>
<xml_diff>
--- a/pvt_list.xlsx
+++ b/pvt_list.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29629"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Dossier LOUMA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_46CBBBEB4BD4E64F51C9DC61FC2C65EABA356C5E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE8C612E-D71E-46E2-9297-A76DBD35E99B}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_46CBBBEB4BD4E64F51C9DC61FC2C65EABA356C5E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C3F5FCC-8EC9-4E26-BE4B-795DB147BE31}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -490,7 +490,7 @@
         <v>5</v>
       </c>
       <c r="C3" s="3">
-        <v>776647468</v>
+        <v>771161412</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15">

</xml_diff>